<commit_message>
Remove __pycache__ files and add data quality improvements
</commit_message>
<xml_diff>
--- a/data/wot_data_definations.xlsx
+++ b/data/wot_data_definations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/satish_byndr/Documents/workspace-py/wot-poc/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947727C3-EE89-E34D-B9A6-DB3B3C92DC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7361450D-B312-DF4C-A649-89A979554468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20020" xr2:uid="{0FCB22E6-9B86-F247-9847-7B38E5BB1147}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="131">
   <si>
     <t>Product Name</t>
   </si>
@@ -544,6 +544,9 @@
 using the project's live services or technology.
 No government partners are included in this
 variable.</t>
+  </si>
+  <si>
+    <t>Archived Source Project Announcement Date</t>
   </si>
 </sst>
 </file>
@@ -643,7 +646,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -669,6 +672,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,7 +1010,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A65D76-1DB5-7E48-ABF0-9B590FA839EE}">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.83203125" style="2" customWidth="1"/>
@@ -1103,7 +1110,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>8</v>
+        <v>130</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>82</v>
@@ -1513,68 +1520,75 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="63" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>92</v>
-      </c>
+    <row r="33" spans="1:5" ht="20" x14ac:dyDescent="0.25">
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="14"/>
     </row>
     <row r="34" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="63" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="168" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="84" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" ht="168" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="84" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E38" s="8" t="s">
         <v>125</v>
       </c>
     </row>

</xml_diff>